<commit_message>
chore: gitignore y BD copiada por build
</commit_message>
<xml_diff>
--- a/netlify/functions/BD participantes.xlsx
+++ b/netlify/functions/BD participantes.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/upmsj/Desktop/UPMSJ /JF/polla/app/antigravity_project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/upmsj/Desktop/UPMSJ /JF/polla/app/pm_project jun/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5EC976A-7E81-6F4E-8813-2C65DCB3339C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3878CD40-6F92-FB41-91C2-A5E5E94C3D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28640" yWindow="2560" windowWidth="28040" windowHeight="17180" xr2:uid="{FA559016-7FAB-0B47-8ABB-CBD3A3CB183F}"/>
+    <workbookView xWindow="-28800" yWindow="2560" windowWidth="28800" windowHeight="17400" xr2:uid="{FA559016-7FAB-0B47-8ABB-CBD3A3CB183F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
   <si>
     <t>ID</t>
   </si>
@@ -227,9 +227,6 @@
     <t>JD0ZTA</t>
   </si>
   <si>
-    <t>Eduardo Vásquez</t>
-  </si>
-  <si>
     <t>Mario Viera</t>
   </si>
   <si>
@@ -239,172 +236,205 @@
     <t>Diego Machado</t>
   </si>
   <si>
-    <t>Participante 1</t>
-  </si>
-  <si>
-    <t>Participante 2</t>
-  </si>
-  <si>
-    <t>Participante 3</t>
-  </si>
-  <si>
-    <t>Participante 4</t>
-  </si>
-  <si>
-    <t>Participante 5</t>
-  </si>
-  <si>
-    <t>Participante 6</t>
-  </si>
-  <si>
-    <t>Participante 7</t>
-  </si>
-  <si>
-    <t>Participante 8</t>
-  </si>
-  <si>
-    <t>Participante 9</t>
-  </si>
-  <si>
-    <t>Participante 10</t>
-  </si>
-  <si>
-    <t>Participante 11</t>
-  </si>
-  <si>
-    <t>Participante 12</t>
-  </si>
-  <si>
-    <t>Participante 13</t>
-  </si>
-  <si>
-    <t>Participante 14</t>
-  </si>
-  <si>
-    <t>Participante 15</t>
-  </si>
-  <si>
-    <t>Participante 16</t>
-  </si>
-  <si>
-    <t>Participante 17</t>
-  </si>
-  <si>
-    <t>Participante 18</t>
-  </si>
-  <si>
-    <t>Participante 19</t>
-  </si>
-  <si>
-    <t>Participante 20</t>
-  </si>
-  <si>
-    <t>Participante 21</t>
-  </si>
-  <si>
-    <t>Participante 22</t>
-  </si>
-  <si>
-    <t>Participante 23</t>
-  </si>
-  <si>
-    <t>Participante 24</t>
-  </si>
-  <si>
-    <t>Participante 25</t>
-  </si>
-  <si>
-    <t>Participante 26</t>
-  </si>
-  <si>
-    <t>Participante 27</t>
-  </si>
-  <si>
-    <t>Participante 28</t>
-  </si>
-  <si>
-    <t>Participante 29</t>
-  </si>
-  <si>
-    <t>Participante 30</t>
-  </si>
-  <si>
-    <t>Participante 31</t>
-  </si>
-  <si>
-    <t>Participante 32</t>
-  </si>
-  <si>
-    <t>Participante 33</t>
-  </si>
-  <si>
-    <t>Participante 34</t>
-  </si>
-  <si>
-    <t>Participante 35</t>
-  </si>
-  <si>
-    <t>Participante 36</t>
-  </si>
-  <si>
-    <t>Participante 37</t>
-  </si>
-  <si>
-    <t>Participante 38</t>
-  </si>
-  <si>
-    <t>Participante 39</t>
-  </si>
-  <si>
-    <t>Participante 40</t>
-  </si>
-  <si>
-    <t>Participante 41</t>
-  </si>
-  <si>
-    <t>Participante 42</t>
-  </si>
-  <si>
-    <t>Participante 43</t>
-  </si>
-  <si>
-    <t>Participante 44</t>
-  </si>
-  <si>
-    <t>Participante 45</t>
-  </si>
-  <si>
-    <t>Participante 46</t>
-  </si>
-  <si>
-    <t>Participante 47</t>
-  </si>
-  <si>
-    <t>Participante 48</t>
-  </si>
-  <si>
-    <t>Participante 49</t>
-  </si>
-  <si>
-    <t>Participante 50</t>
-  </si>
-  <si>
-    <t>Participante 51</t>
-  </si>
-  <si>
-    <t>Participante 52</t>
-  </si>
-  <si>
-    <t>Participante 53</t>
-  </si>
-  <si>
-    <t>Participante 54</t>
-  </si>
-  <si>
-    <t>Participante 55</t>
-  </si>
-  <si>
-    <t>Participante 56</t>
+    <t>Gabriel Larco</t>
+  </si>
+  <si>
+    <t>Gabriel Cepeda</t>
+  </si>
+  <si>
+    <t>Daniel Larco</t>
+  </si>
+  <si>
+    <t>Facundo Larco</t>
+  </si>
+  <si>
+    <t>Tomás Larco</t>
+  </si>
+  <si>
+    <t>Andrés Camelos</t>
+  </si>
+  <si>
+    <t>Cristina Torres</t>
+  </si>
+  <si>
+    <t>Nicolás Vásquez</t>
+  </si>
+  <si>
+    <t>Roberto Mucarsel H</t>
+  </si>
+  <si>
+    <t>Robert Mucarsel B</t>
+  </si>
+  <si>
+    <t>Ariel Mucarsel B</t>
+  </si>
+  <si>
+    <t>Benja Mucarsel B</t>
+  </si>
+  <si>
+    <t>Hipa Vásquez</t>
+  </si>
+  <si>
+    <t>Ramiro Almeida</t>
+  </si>
+  <si>
+    <t>Ronny Almeida</t>
+  </si>
+  <si>
+    <t>Carlos Almeida</t>
+  </si>
+  <si>
+    <t>José Luis Zavala</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carmen Falcones </t>
+  </si>
+  <si>
+    <t>Margoth Jacobowitz</t>
+  </si>
+  <si>
+    <t>Antonio Torres</t>
+  </si>
+  <si>
+    <t>Bryan Montalvo</t>
+  </si>
+  <si>
+    <t>Irene Vásquez</t>
+  </si>
+  <si>
+    <t>Pepe Vaca</t>
+  </si>
+  <si>
+    <t>Eduardo M Vásquez</t>
+  </si>
+  <si>
+    <t>Eduardo J Vásquez</t>
+  </si>
+  <si>
+    <t>Daniel Guevara</t>
+  </si>
+  <si>
+    <t>Sergio Montalvo</t>
+  </si>
+  <si>
+    <t>Abraham Loja</t>
+  </si>
+  <si>
+    <t>Gonzalo Vásquez</t>
+  </si>
+  <si>
+    <t>Edgar Moreno</t>
+  </si>
+  <si>
+    <t>Alex Moreno</t>
+  </si>
+  <si>
+    <t>Luis Moreno</t>
+  </si>
+  <si>
+    <t>Paco Ortiz</t>
+  </si>
+  <si>
+    <t>Ma José Sánchez</t>
+  </si>
+  <si>
+    <t>Andrés Ávalos</t>
+  </si>
+  <si>
+    <t>Carlos Castro</t>
+  </si>
+  <si>
+    <t>Doménica Larrea</t>
+  </si>
+  <si>
+    <t>Mario Viera C</t>
+  </si>
+  <si>
+    <t>Katty Naranjo</t>
+  </si>
+  <si>
+    <t>Paz Haro</t>
+  </si>
+  <si>
+    <t>Jonathan Loor</t>
+  </si>
+  <si>
+    <t>Jaime Brito</t>
+  </si>
+  <si>
+    <t>Robert Jiménez</t>
+  </si>
+  <si>
+    <t>Johnny Guevara</t>
+  </si>
+  <si>
+    <t>Martín Buitrón</t>
+  </si>
+  <si>
+    <t>Antony Ramos</t>
+  </si>
+  <si>
+    <t>Edison Orbe</t>
+  </si>
+  <si>
+    <t>Ramiro O Vallejo</t>
+  </si>
+  <si>
+    <t>Ramiro A Vallejo</t>
+  </si>
+  <si>
+    <t>Roberto Peñafiel</t>
+  </si>
+  <si>
+    <t>J29QPX</t>
+  </si>
+  <si>
+    <t>8PV3KZ</t>
+  </si>
+  <si>
+    <t>Jeffry Trujillo</t>
+  </si>
+  <si>
+    <t>Fabián Procel</t>
+  </si>
+  <si>
+    <t>UHOAFN</t>
+  </si>
+  <si>
+    <t>Jonathan Vásquez</t>
+  </si>
+  <si>
+    <t>G9DBE7</t>
+  </si>
+  <si>
+    <t>Carlos F Castro</t>
+  </si>
+  <si>
+    <t>Sebastián Larco</t>
+  </si>
+  <si>
+    <t>José Viera</t>
+  </si>
+  <si>
+    <t>Kevin Puga</t>
+  </si>
+  <si>
+    <t>DX9TWC</t>
+  </si>
+  <si>
+    <t>André Encalada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christian Guevara </t>
+  </si>
+  <si>
+    <t>Javier García</t>
+  </si>
+  <si>
+    <t>Oscar Arteaga</t>
+  </si>
+  <si>
+    <t>Hernán Espinoza</t>
   </si>
 </sst>
 </file>
@@ -459,7 +489,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -469,6 +499,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -804,12 +837,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7136B2E9-7B51-874A-BFBE-4CAB6091C4C3}">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
     <col min="3" max="3" width="24.5" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -828,7 +862,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
@@ -839,7 +873,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>4</v>
@@ -850,7 +884,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
@@ -861,7 +895,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>6</v>
@@ -872,7 +906,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>7</v>
@@ -883,7 +917,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>68</v>
+        <v>124</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
@@ -894,7 +928,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>9</v>
@@ -905,7 +939,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>70</v>
+        <v>129</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>10</v>
@@ -916,7 +950,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>11</v>
@@ -927,7 +961,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>72</v>
+        <v>128</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>12</v>
@@ -938,7 +972,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>13</v>
@@ -949,7 +983,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>14</v>
@@ -960,7 +994,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>15</v>
@@ -971,7 +1005,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>16</v>
@@ -982,7 +1016,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>17</v>
@@ -993,7 +1027,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>18</v>
@@ -1004,7 +1038,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>19</v>
@@ -1015,7 +1049,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>20</v>
@@ -1026,7 +1060,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>21</v>
@@ -1037,7 +1071,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>22</v>
@@ -1048,7 +1082,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>23</v>
@@ -1059,7 +1093,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>84</v>
+        <v>131</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>24</v>
@@ -1070,7 +1104,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>25</v>
@@ -1081,7 +1115,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>26</v>
@@ -1092,7 +1126,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>27</v>
@@ -1103,7 +1137,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>28</v>
@@ -1114,7 +1148,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>29</v>
@@ -1125,7 +1159,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>30</v>
@@ -1136,7 +1170,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>31</v>
@@ -1147,7 +1181,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>32</v>
@@ -1158,7 +1192,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>33</v>
@@ -1169,7 +1203,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>34</v>
@@ -1180,7 +1214,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>95</v>
+        <v>130</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>35</v>
@@ -1191,7 +1225,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>36</v>
@@ -1202,7 +1236,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>37</v>
@@ -1213,7 +1247,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>38</v>
@@ -1224,7 +1258,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>39</v>
@@ -1235,7 +1269,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>40</v>
@@ -1246,7 +1280,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>41</v>
@@ -1257,7 +1291,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>42</v>
@@ -1268,7 +1302,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>43</v>
@@ -1279,7 +1313,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>44</v>
@@ -1290,7 +1324,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>45</v>
@@ -1301,7 +1335,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>46</v>
@@ -1312,7 +1346,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>47</v>
@@ -1323,7 +1357,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>48</v>
@@ -1334,154 +1368,236 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
         <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
         <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
         <v>58</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
         <v>59</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
         <v>60</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>62</v>
       </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="2">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="2">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="2">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D64" s="2"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="2">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D65" s="2"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="2">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D66" s="2"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D67" s="2"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D68" s="2"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D69" s="2"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D70" s="2"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D71" s="2"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D72" s="2"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D73" s="2"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D74" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>